<commit_message>
perfil: tasa de hora no ejecutada por servicio
</commit_message>
<xml_diff>
--- a/DICCIONARIO_DE_DATOS_CONSULTA_EXTERNA_2015_2022_0.xlsx
+++ b/DICCIONARIO_DE_DATOS_CONSULTA_EXTERNA_2015_2022_0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeanpierre\Desktop\proyectos personales\proyecto_essalud\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E812E4-6AB1-41C3-99E4-143FA635A01F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B586F9-A454-4410-8734-E4307B2FB1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D0ABD994-8406-468F-BE4E-4AECADAB2CE5}"/>
   </bookViews>
@@ -160,7 +160,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +180,14 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -236,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -253,12 +261,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,14 +594,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -638,7 +647,7 @@
       <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>28</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -656,7 +665,7 @@
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -672,7 +681,7 @@
       <c r="A8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -688,7 +697,7 @@
       <c r="A9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C9" s="6" t="s">
@@ -704,7 +713,7 @@
       <c r="A10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -720,7 +729,7 @@
       <c r="A11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>36</v>
       </c>
       <c r="C11" s="6"/>
@@ -732,7 +741,7 @@
       <c r="A12" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="6" t="s">
@@ -748,7 +757,7 @@
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="6" t="s">
@@ -757,7 +766,7 @@
       <c r="D13" s="4">
         <v>20</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="4"/>
@@ -766,7 +775,7 @@
       <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>39</v>
       </c>
       <c r="C14" s="6" t="s">
@@ -775,7 +784,7 @@
       <c r="D14" s="4">
         <v>100</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="4"/>
@@ -784,7 +793,7 @@
       <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="8" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="6" t="s">
@@ -793,16 +802,16 @@
       <c r="D15" s="4">
         <v>100</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="6" t="s">
@@ -811,7 +820,7 @@
       <c r="D16" s="4">
         <v>6</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="4"/>
@@ -820,7 +829,7 @@
       <c r="A17" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="6" t="s">
@@ -829,8 +838,8 @@
       <c r="D17" s="4">
         <v>8</v>
       </c>
-      <c r="E17" s="9"/>
-      <c r="F17" s="4" t="s">
+      <c r="E17" s="8"/>
+      <c r="F17" s="10" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>